<commit_message>
fix: align scenario DCF IPO proceeds
</commit_message>
<xml_diff>
--- a/model/MWG_DMX_IPO_SOTP_Model.xlsx
+++ b/model/MWG_DMX_IPO_SOTP_Model.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Cover'!$B$2:$J$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Q1_Actuals'!$A$4:$J$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Assumptions'!$A$10:$K$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Checks'!$A$4:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Checks'!$A$4:$H$25</definedName>
   </definedNames>
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>46216.91675925926</v>
+        <v>46216.94168981481</v>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
@@ -2669,7 +2669,7 @@
     <row r="24" ht="24" customHeight="1">
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>6. Do earnings, working capital, cash and retained earnings reconcile across the three statements?</t>
+          <t>6. Do earnings, working capital, cash and retained earnings residuals reconcile across the three statements?</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>NPAT-to-CFO, cash, retained earnings and normalization</t>
+          <t>NPAT-to-CFO, cash, retained-earnings residual and normalization</t>
         </is>
       </c>
       <c r="D32" s="16" t="n"/>
@@ -6452,7 +6452,7 @@
       <c r="D38" s="153" t="n"/>
       <c r="E38" s="153" t="n"/>
       <c r="F38" s="147">
-        <f>F37-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$E$21-Assumptions!$E$22+Assumptions!$E$20</f>
+        <f>F37-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$E$21-Assumptions!$E$22+Assumptions!$E$20</f>
         <v/>
       </c>
       <c r="H38" s="153" t="n"/>
@@ -6460,7 +6460,7 @@
       <c r="J38" s="153" t="n"/>
       <c r="K38" s="153" t="n"/>
       <c r="L38" s="147">
-        <f>L37-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20</f>
+        <f>L37-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20</f>
         <v/>
       </c>
       <c r="N38" s="153" t="n"/>
@@ -6468,7 +6468,7 @@
       <c r="P38" s="153" t="n"/>
       <c r="Q38" s="153" t="n"/>
       <c r="R38" s="147">
-        <f>R37-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$G$21-Assumptions!$G$22+Assumptions!$G$20</f>
+        <f>R37-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$G$21-Assumptions!$G$22+Assumptions!$G$20</f>
         <v/>
       </c>
     </row>
@@ -6559,23 +6559,23 @@
         <v>0.1</v>
       </c>
       <c r="C46" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B46-C$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B46-C$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="D46" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B46-D$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B46-D$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="E46" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B46-E$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B46-E$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="F46" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B46-F$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B46-F$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="G46" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B46-G$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B46)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B46-G$45)/(1+$B46)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="J46" s="159" t="n">
@@ -6603,23 +6603,23 @@
         <v>0.11</v>
       </c>
       <c r="C47" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B47-C$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B47-C$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="D47" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B47-D$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B47-D$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="E47" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B47-E$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B47-E$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="F47" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B47-F$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B47-F$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="G47" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B47-G$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B47)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B47-G$45)/(1+$B47)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="J47" s="159" t="n">
@@ -6647,23 +6647,23 @@
         <v>0.12</v>
       </c>
       <c r="C48" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B48-C$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B48-C$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="D48" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B48-D$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B48-D$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="E48" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B48-E$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B48-E$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="F48" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B48-F$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B48-F$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="G48" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B48-G$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B48)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B48-G$45)/(1+$B48)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="J48" s="159" t="n">
@@ -6691,23 +6691,23 @@
         <v>0.13</v>
       </c>
       <c r="C49" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B49-C$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B49-C$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="D49" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B49-D$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B49-D$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="E49" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B49-E$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B49-E$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="F49" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B49-F$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B49-F$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="G49" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B49-G$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B49)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B49-G$45)/(1+$B49)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="J49" s="159" t="n">
@@ -6735,23 +6735,23 @@
         <v>0.14</v>
       </c>
       <c r="C50" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B50-C$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+C$45)/($B50-C$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="D50" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B50-D$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+D$45)/($B50-D$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="E50" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B50-E$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+E$45)/($B50-E$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="F50" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B50-F$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+F$45)/($B50-F$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="G50" s="158">
-        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B50-G$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
+        <f>(SUMPRODUCT($H$29:$L$29,1/(1+$B50)^{0.5,1.5,2.5,3.5,4.5})+$L$29*(1+G$45)/($B50-G$45)/(1+$B50)^4.5-Q1_Actuals!D36+Q1_Actuals!D25+Q1_Actuals!D26+Q1_Actuals!D27+IPO_Bridge!$D$20-Assumptions!$F$21-Assumptions!$F$22+Assumptions!$F$20)*1000/IPO_Bridge!D11</f>
         <v/>
       </c>
       <c r="J50" s="159" t="n">
@@ -6829,7 +6829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -6948,7 +6948,7 @@
         </is>
       </c>
       <c r="J5" s="164">
-        <f>COUNTIFS(C5:C24,"Critical",G5:G24,"FAIL*")</f>
+        <f>COUNTIFS(C5:C25,"Critical",G5:G25,"FAIL*")</f>
         <v/>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
         </is>
       </c>
       <c r="J6" s="164">
-        <f>COUNTIF(G5:G24,"WARN*")</f>
+        <f>COUNTIF(G5:G25,"WARN*")</f>
         <v/>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
         <v>0.01</v>
       </c>
       <c r="F15" s="161">
-        <f>ABS(DMX_Valuation!K22-IPO_Bridge!D19)</f>
+        <f>ABS(DMX_Valuation!K22-IPO_Bridge!D20)</f>
         <v/>
       </c>
       <c r="G15" s="162">
@@ -7710,13 +7710,51 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="95" t="inlineStr">
+        <is>
+          <t>CHK_SCENARIO_BASE_DCF_MATCH</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>Scenarios</t>
+        </is>
+      </c>
+      <c r="C25" s="160" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D25" s="28" t="inlineStr">
+        <is>
+          <t>Base scenario DMX equity value equals DMX_Valuation when active scenario is Base</t>
+        </is>
+      </c>
+      <c r="E25" s="39" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F25" s="161">
+        <f>IF(Assumptions!C4="Base",ABS(Scenarios!L38-DMX_Valuation!K23),0)</f>
+        <v/>
+      </c>
+      <c r="G25" s="162">
+        <f>IF(F25&lt;=E25,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="H25" s="28" t="inlineStr">
+        <is>
+          <t>Prevents the independent scenario block from omitting pro forma net IPO proceeds or other EV-to-equity bridge items</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H24"/>
+  <autoFilter ref="A4:H25"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G24">
+  <conditionalFormatting sqref="G5:G25">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LEFT(G5,4)="PASS"</formula>
     </cfRule>
@@ -12315,7 +12353,7 @@
     <row r="2" ht="23" customHeight="1">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>Q1 2026 earnings-to-cash, cash roll-forward, FY2025 retained earnings, normalization and IPO pro forma controls.</t>
+          <t>Q1 2026 earnings-to-cash, cash roll-forward, FY2025 retained-earnings residual reconciliation, normalization and IPO pro forma controls.</t>
         </is>
       </c>
     </row>
@@ -12332,7 +12370,7 @@
       </c>
       <c r="K4" s="68" t="inlineStr">
         <is>
-          <t>Retained earnings · FY2025</t>
+          <t>Retained earnings residual · FY2025</t>
         </is>
       </c>
     </row>
@@ -12433,7 +12471,7 @@
       </c>
       <c r="K8" s="61" t="inlineStr">
         <is>
-          <t>Capitalisation / other equity movements</t>
+          <t>Residual: capitalisation / other equity movements</t>
         </is>
       </c>
       <c r="L8" s="70" t="n">
@@ -12569,7 +12607,7 @@
       </c>
       <c r="K13" s="73" t="inlineStr">
         <is>
-          <t>FY2025 residual captures the disclosed capital restructuring and other equity movements; it is not treated as an operating adjustment.</t>
+          <t>Residual reconciliation only: detailed statement-of-changes-in-equity lines are not fully available in the public case set. FY2025 residual captures the disclosed capital restructuring and other equity movements; it is not treated as an operating adjustment.</t>
         </is>
       </c>
     </row>

</xml_diff>